<commit_message>
Master file: ATIP stays single-owner (owner decision)
The owner decided on 2026-10-26 to keep ATIP single-owner, in line with the
owner-only gate of #11, so the consolidated prompt's multi-user phases are not
planned. The master file records the decision: the multi-user target
architecture is marked "not adopted", the per-user review rows (registration,
roles, per-user holdings and Dhan accounts, personalization, per-user
execution, their tests) say "Not planned", roadmap R9 is dropped, and R10
becomes deploying the single-owner ATIP behind the owner gate. The
/api/orders read leak stays listed as latent (enterprise mode only, R11).
Rows P1 and P7 note that master is green again since #16. The workbook is
rebuilt from the markdown.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQAcu5VWVUXxeTxHUKWC9Z
</commit_message>
<xml_diff>
--- a/docs/master/ATIP_MASTER_FILE_2026-10-26.xlsx
+++ b/docs/master/ATIP_MASTER_FILE_2026-10-26.xlsx
@@ -49,7 +49,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Sim_Geometry'!$A$1:$K$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Sim_Policies'!$A$1:$K$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Sim_Required_Edge'!$A$1:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Roadmap'!$A$1:$E$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Roadmap'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26286,7 +26286,7 @@
       </c>
       <c r="K335" s="2" t="inlineStr">
         <is>
-          <t>Both fixes exist in PR #16 and are carried in this PR so its CI can go green</t>
+          <t>Both fixes merged with #16; master is green again from run 169</t>
         </is>
       </c>
       <c r="L335" s="2" t="inlineStr"/>
@@ -26430,7 +26430,7 @@
       </c>
       <c r="K338" s="2" t="inlineStr">
         <is>
-          <t>Decide on 6.1 (1) first</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
       <c r="L338" s="2" t="inlineStr"/>
@@ -26478,7 +26478,7 @@
       </c>
       <c r="K339" s="2" t="inlineStr">
         <is>
-          <t>No functional tests of login, logout, refresh or expiry; set Secure cookies on any hosted install</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26). The owner signs in through the central bkesari.com gate of PR #11 (dashboard/owner_gate.py there)</t>
         </is>
       </c>
       <c r="L339" s="2" t="inlineStr"/>
@@ -26622,7 +26622,7 @@
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>Map ADMIN → SUPER_ADMIN of tenant default, USER → TRADER or VIEWER</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr"/>
@@ -26670,7 +26670,7 @@
       </c>
       <c r="K343" s="2" t="inlineStr">
         <is>
-          <t>X-ATIP-Token is one install-wide secret embedded in every page (dashboard/server.py:860-862), not per user</t>
+          <t>One install-wide X-ATIP-Token fits a single owner: keep it secret and rotate it after any leak (W40 runbook)</t>
         </is>
       </c>
       <c r="L343" s="2" t="inlineStr"/>
@@ -26718,7 +26718,7 @@
       </c>
       <c r="K344" s="2" t="inlineStr">
         <is>
-          <t>Leak: GET /api/orders (and /pending, /baskets, /sip) needs only execution:read (authz.py:138), which is in neither PAPER_BOOK (:152) nor FILTER_PREFIX (:175), so any tenant's VIEWER reads the owner's order rules; / embeds the owner's portfolio. No test covers cross-tenant 404s or filtering</t>
+          <t>Latent, enterprise mode only: GET /api/orders (and /pending, /baskets, /sip) needs only execution:read (enterprise/authz.py:138), in neither PAPER_BOOK (:152) nor FILTER_PREFIX (:175). Single-owner keeps enterprise mode off; fix it before it is ever switched on</t>
         </is>
       </c>
       <c r="L344" s="2" t="inlineStr"/>
@@ -26766,7 +26766,7 @@
       </c>
       <c r="K345" s="2" t="inlineStr">
         <is>
-          <t>Add owner scoping per table, or keep one user per tenant</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
       <c r="L345" s="2" t="inlineStr"/>
@@ -26814,7 +26814,7 @@
       </c>
       <c r="K346" s="2" t="inlineStr">
         <is>
-          <t>Only read-only connectors use it (brokers/registry.py:37-72); orders, market data and the strategy use the owner's global client (orders/broker.py:157,272); a default-tenant user without a vault entry silently gets the owner's credentials (enterprise/vault.py:184-187)</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26): the owner's credentials stay in config.json / the vault</t>
         </is>
       </c>
       <c r="L346" s="2" t="inlineStr"/>
@@ -26910,7 +26910,7 @@
       </c>
       <c r="K348" s="2" t="inlineStr">
         <is>
-          <t>No per-user layout, widgets or theme; the main page is rendered without knowing the user (dashboard/server.py:1339-1341)</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
       <c r="L348" s="2" t="inlineStr"/>
@@ -26958,7 +26958,7 @@
       </c>
       <c r="K349" s="2" t="inlineStr">
         <is>
-          <t>No test that a non-admin is refused</t>
+          <t>Not applicable with one owner</t>
         </is>
       </c>
       <c r="L349" s="2" t="inlineStr"/>
@@ -27294,7 +27294,7 @@
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>Needs user / tenant columns, per-user config and per-user broker routing, after 6.1 (1)</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr"/>
@@ -27486,7 +27486,7 @@
       </c>
       <c r="K360" s="2" t="inlineStr">
         <is>
-          <t>Write them once 6.1 (1) is decided</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26); PR #11 tests the owner gate (tests/test_owner_gate.py there)</t>
         </is>
       </c>
       <c r="L360" s="2" t="inlineStr"/>
@@ -27534,7 +27534,7 @@
       </c>
       <c r="K361" s="2" t="inlineStr">
         <is>
-          <t>Add cross-tenant 404 / filter tests, including /api/orders</t>
+          <t>Only if enterprise mode is ever switched on (with the /api/orders fix, row P3)</t>
         </is>
       </c>
       <c r="L361" s="2" t="inlineStr"/>
@@ -27582,7 +27582,7 @@
       </c>
       <c r="K362" s="2" t="inlineStr">
         <is>
-          <t>After P3 / P5</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
       <c r="L362" s="2" t="inlineStr"/>
@@ -27616,9 +27616,9 @@
         </is>
       </c>
       <c r="F363" s="2" t="inlineStr"/>
-      <c r="G363" s="7" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="G363" s="4" t="inlineStr">
+        <is>
+          <t>PRESENT</t>
         </is>
       </c>
       <c r="H363" s="2" t="inlineStr"/>
@@ -27630,7 +27630,7 @@
       </c>
       <c r="K363" s="2" t="inlineStr">
         <is>
-          <t>master is red on the two tests in row P1</t>
+          <t>master green from run 169 (#16); this branch 1,578 passed, 0 failed</t>
         </is>
       </c>
       <c r="L363" s="2" t="inlineStr"/>
@@ -27774,7 +27774,7 @@
       </c>
       <c r="K366" s="2" t="inlineStr">
         <is>
-          <t>Add a read-only "Aggressive positions" panel and API</t>
+          <t>Single-owner: the existing dashboard behind the owner gate. Still worth adding: a read-only "Aggressive positions" panel and API</t>
         </is>
       </c>
       <c r="L366" s="2" t="inlineStr"/>
@@ -28955,7 +28955,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Both fixes exist in PR #16 and are carried in this PR so its CI can go green</t>
+          <t>Both fixes merged with #16; master is green again from run 169</t>
         </is>
       </c>
     </row>
@@ -29051,7 +29051,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Decide on 6.1 (1) first</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
     </row>
@@ -29083,7 +29083,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>No functional tests of login, logout, refresh or expiry; set Secure cookies on any hosted install</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26). The owner signs in through the central bkesari.com gate of PR #11 (dashboard/owner_gate.py there)</t>
         </is>
       </c>
     </row>
@@ -29179,7 +29179,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Map ADMIN → SUPER_ADMIN of tenant default, USER → TRADER or VIEWER</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
     </row>
@@ -29211,7 +29211,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>X-ATIP-Token is one install-wide secret embedded in every page (dashboard/server.py:860-862), not per user</t>
+          <t>One install-wide X-ATIP-Token fits a single owner: keep it secret and rotate it after any leak (W40 runbook)</t>
         </is>
       </c>
     </row>
@@ -29243,7 +29243,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Leak: GET /api/orders (and /pending, /baskets, /sip) needs only execution:read (authz.py:138), which is in neither PAPER_BOOK (:152) nor FILTER_PREFIX (:175), so any tenant's VIEWER reads the owner's order rules; / embeds the owner's portfolio. No test covers cross-tenant 404s or filtering</t>
+          <t>Latent, enterprise mode only: GET /api/orders (and /pending, /baskets, /sip) needs only execution:read (enterprise/authz.py:138), in neither PAPER_BOOK (:152) nor FILTER_PREFIX (:175). Single-owner keeps enterprise mode off; fix it before it is ever switched on</t>
         </is>
       </c>
     </row>
@@ -29275,7 +29275,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Add owner scoping per table, or keep one user per tenant</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Only read-only connectors use it (brokers/registry.py:37-72); orders, market data and the strategy use the owner's global client (orders/broker.py:157,272); a default-tenant user without a vault entry silently gets the owner's credentials (enterprise/vault.py:184-187)</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26): the owner's credentials stay in config.json / the vault</t>
         </is>
       </c>
     </row>
@@ -29371,7 +29371,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>No per-user layout, widgets or theme; the main page is rendered without knowing the user (dashboard/server.py:1339-1341)</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
     </row>
@@ -29403,7 +29403,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>No test that a non-admin is refused</t>
+          <t>Not applicable with one owner</t>
         </is>
       </c>
     </row>
@@ -29627,7 +29627,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Needs user / tenant columns, per-user config and per-user broker routing, after 6.1 (1)</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
     </row>
@@ -29755,7 +29755,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Write them once 6.1 (1) is decided</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26); PR #11 tests the owner gate (tests/test_owner_gate.py there)</t>
         </is>
       </c>
     </row>
@@ -29787,7 +29787,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Add cross-tenant 404 / filter tests, including /api/orders</t>
+          <t>Only if enterprise mode is ever switched on (with the /api/orders fix, row P3)</t>
         </is>
       </c>
     </row>
@@ -29819,7 +29819,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>After P3 / P5</t>
+          <t>Not planned: ATIP stays single-owner (owner decision 2026-10-26)</t>
         </is>
       </c>
     </row>
@@ -29839,9 +29839,9 @@
           <t>Full regression stays green</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>PRESENT</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -29851,7 +29851,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>master is red on the two tests in row P1</t>
+          <t>master green from run 169 (#16); this branch 1,578 passed, 0 failed</t>
         </is>
       </c>
     </row>
@@ -29947,7 +29947,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Add a read-only "Aggressive positions" panel and API</t>
+          <t>Single-owner: the existing dashboard behind the owner gate. Still worth adding: a read-only "Aggressive positions" panel and API</t>
         </is>
       </c>
     </row>
@@ -30887,7 +30887,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>1. Fixed (owner-approved, 2026-10-26): MRI was read the wrong way round at the +6% runner checkpoint. The score engine scores MRI so that higher is more bullish (scores/engine.py:470-487), and the signal engine sells on low MRI (scores/engine.py:807). But Momentum.composite inverted MRI as a risk measure, so strong momentum pushed a runner toward exit and weak momentum toward holding. MRI now enters as it is (strategy/aggressive.py:198-199). The test fixtures are mirrored, so every existing result is unchanged, and test_mri_counts_as_strength_the_way_the_score_engine_reads_it pins the direction against determine_signal. 2. Index names disagree across documents. The code defines VPI as Volatility-Potential and SPI as Stability Profit. The strategy library and the formulas workbook call them "value/profit" and "stock/sector strength". §4 fixes the canonical meanings from the code. 3. The consolidated prompt's aggressive-strategy logic (phases 4, 6, 8, 13) is already built and tested. Nothing scheduled it: exits ran only when python -m strategy.live --manage was run by hand. Scheduled (owner-approved, 2026-10-26): a management pass now runs every manage_interval_minutes (default 2) from 09:15 to 15:30 on trading days while a position is open. Unattended, it never sells a position through a broker other than the one it was opened with (PAPER vs LIVE). The multi-user phases (3, 5, 9, 10, 12) are only partly in place, and open PR #11 (owner-only gate) points the other way. See §6 before any new implementation starts.</t>
+          <t>1. Fixed (owner-approved, 2026-10-26): MRI was read the wrong way round at the +6% runner checkpoint. The score engine scores MRI so that higher is more bullish (scores/engine.py:470-487), and the signal engine sells on low MRI (scores/engine.py:807). But Momentum.composite inverted MRI as a risk measure, so strong momentum pushed a runner toward exit and weak momentum toward holding. MRI now enters as it is (strategy/aggressive.py:198-199). The test fixtures are mirrored, so every existing result is unchanged, and test_mri_counts_as_strength_the_way_the_score_engine_reads_it pins the direction against determine_signal. 2. Index names disagree across documents. The code defines VPI as Volatility-Potential and SPI as Stability Profit. The strategy library and the formulas workbook call them "value/profit" and "stock/sector strength". §4 fixes the canonical meanings from the code. 3. The consolidated prompt's aggressive-strategy logic (phases 4, 6, 8, 13) is already built and tested. Nothing scheduled it: exits ran only when python -m strategy.live --manage was run by hand. Scheduled (owner-approved, 2026-10-26): a management pass now runs every manage_interval_minutes (default 2) from 09:15 to 15:30 on trading days while a position is open. Unattended, it never sells a position through a broker other than the one it was opened with (PAPER vs LIVE). Decided 2026-10-26: ATIP stays single-owner, in line with PR #11's owner-only gate, so the prompt's multi-user phases (3, 5 and the per-user parts of 7 and 9) are not planned. See §6.</t>
         </is>
       </c>
     </row>
@@ -34860,7 +34860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -35121,22 +35121,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Multi-user items from §6 (only if a multi-user product is wanted)</t>
+          <t>Dropped 2026-10-26: multi-user items from §6. ATIP stays single-owner (owner decision)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Consolidated-prompt phases 3, 5, 9, 10</t>
+          <t>Consolidated-prompt phases 3, 5 and the per-user parts of 7 and 9</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -35153,12 +35153,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Deploy to test.bkesari.com/dhan once hosting and secrets are decided</t>
+          <t>Deploy the single-owner ATIP to test.bkesari.com behind the owner gate (PR #11), with the base-path fix, once hosting and secrets are decided</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Consolidated-prompt phase 10</t>
+          <t>Consolidated-prompt phase 10, decision 6.1 (3)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -35167,8 +35167,35 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Close the latent /api/orders read leak in enterprise/authz.py (enterprise mode only)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Review row P3; matters only if enterprise mode is ever switched on</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
+  <autoFilter ref="A1:E12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>